<commit_message>
Adding timeslice for VAR_FOUT
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_EST/ReportDefs_vervestacks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9080BAB-9E79-43E9-804D-92CCE048C677}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D40D2B4-B86E-4418-A2A5-5EAD31622E9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap_OLD" sheetId="70" r:id="rId1"/>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="860" uniqueCount="423">
   <si>
     <t>Unit</t>
   </si>
@@ -1895,17 +1895,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6A01595-4651-4682-AE2C-4C2356B80CEF}">
   <dimension ref="A1:U60"/>
-  <sheetFormatPr defaultColWidth="14.73046875" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="14.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="19.86328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.59765625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.59765625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.59765625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="1.73046875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="1.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="4.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21">
@@ -2303,11 +2303,11 @@
         <v>vstacks_s3p3v3_d~0004</v>
       </c>
       <c r="C14" t="str">
-        <f t="shared" si="1"/>
+        <f>H14</f>
         <v>b 2 deg (50%).d9d</v>
       </c>
       <c r="H14" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TEXTJOIN(".",TRUE,I14:J14)</f>
         <v>b 2 deg (50%).d9d</v>
       </c>
       <c r="I14" t="str">
@@ -3927,22 +3927,22 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10ADB714-E6AA-4E3E-B77B-62B65BA0E218}">
   <dimension ref="A1:G66"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.86328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.06640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="15.265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.46484375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.53125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="17.25" thickBot="1">
+    <row r="1" spans="1:7" ht="18" thickBot="1">
       <c r="A1" s="5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15" thickTop="1" thickBot="1">
+    <row r="2" spans="1:7" ht="16.5" thickTop="1" thickBot="1">
       <c r="A2" s="6" t="s">
         <v>53</v>
       </c>
@@ -4734,16 +4734,16 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE3245E1-8745-41DD-8AE6-2F4FA19D9F1C}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.73046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.73046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.86328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.59765625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.73046875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -4786,9 +4786,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="4" max="4" width="10.86328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -4831,14 +4831,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr codeName="Sheet31"/>
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.1328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.73046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.86328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.73046875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="5" bestFit="1" customWidth="1"/>
@@ -4944,27 +4944,27 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet11"/>
   <dimension ref="B1:X75"/>
-  <sheetFormatPr defaultColWidth="14.73046875" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="14.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="2.73046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.86328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.59765625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.59765625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.59765625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.53125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.19921875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.06640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="6.53125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="2.73046875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.33203125" customWidth="1"/>
-    <col min="23" max="23" width="2.73046875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="13.06640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.28515625" customWidth="1"/>
+    <col min="23" max="23" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:24">
@@ -7764,38 +7764,38 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet19"/>
   <dimension ref="A1:U22"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.86328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.73046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="16.86328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.59765625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.86328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.73046875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.73046875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.59765625" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="8.73046875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.265625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.1328125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="4.53125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="22.59765625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="6.53125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.59765625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="2.1328125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.86328125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="14.3984375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.73046875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="107.73046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="4.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="2.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="107.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="17.25" thickBot="1">
+    <row r="1" spans="1:21" ht="18" thickBot="1">
       <c r="A1" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="15" thickTop="1" thickBot="1">
+    <row r="2" spans="1:21" ht="16.5" thickTop="1" thickBot="1">
       <c r="A2" s="6" t="s">
         <v>11</v>
       </c>
@@ -7907,6 +7907,9 @@
       </c>
       <c r="N5" t="s">
         <v>81</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>118</v>
       </c>
       <c r="T5" s="3" t="s">
         <v>44</v>
@@ -8241,17 +8244,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68A8EC7F-95E3-4526-8B78-C58A96098159}">
   <dimension ref="C1:K3"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="3" width="17.53125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.1328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.19921875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.19921875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.46484375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="3:11">
@@ -8321,17 +8324,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31D44EBE-400A-4EA2-9DA1-076783A77DFC}">
   <dimension ref="A3:S23"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="19" width="19.265625" customWidth="1"/>
+    <col min="1" max="19" width="19.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:19" ht="17.25" thickBot="1">
+    <row r="3" spans="1:19" ht="18" thickBot="1">
       <c r="A3" s="5" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="15" thickTop="1" thickBot="1">
+    <row r="4" spans="1:19" ht="16.5" thickTop="1" thickBot="1">
       <c r="A4" s="6" t="s">
         <v>11</v>
       </c>
@@ -8434,12 +8437,12 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="17.25" thickBot="1">
+    <row r="10" spans="1:19" ht="18" thickBot="1">
       <c r="A10" s="5" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="15" thickTop="1" thickBot="1">
+    <row r="11" spans="1:19" ht="16.5" thickTop="1" thickBot="1">
       <c r="A11" s="6" t="s">
         <v>11</v>
       </c>
@@ -8681,10 +8684,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:C47"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="11.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9116,7 +9119,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3E766D8-7F73-4A5A-98A5-9C85D527817F}">
   <dimension ref="A1:C35"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
   </cols>
@@ -9440,11 +9443,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.59765625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.1328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.3984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9571,11 +9574,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32957E82-8232-40A9-A839-CC5F79005B92}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.1328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.19921875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">

</xml_diff>